<commit_message>
Added updated project proposal, risk analysis and Software Requirements specificaiton
</commit_message>
<xml_diff>
--- a/Risk Analysis.xlsx
+++ b/Risk Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tewaka-my.sharepoint.com/personal/rcw0085_arastudent_ac_nz/Documents/Courses/Software Development Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{0B148BE9-2A3B-4DD4-96F0-BC10C214FAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF0ED1B4-A310-44E8-89F8-F544304D1D22}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="8_{0B148BE9-2A3B-4DD4-96F0-BC10C214FAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F97E139C-634E-4DE8-9D9F-42B65F08744C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Risks" sheetId="18" r:id="rId1"/>
@@ -257,17 +257,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
   <si>
     <t>Triggers</t>
   </si>
   <si>
-    <t>Date:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative, Project, and/or Engagement: </t>
-  </si>
-  <si>
     <t>Contingency</t>
   </si>
   <si>
@@ -301,16 +295,97 @@
     <t>Risk Assessment Template</t>
   </si>
   <si>
-    <t xml:space="preserve">Organisation: </t>
-  </si>
-  <si>
-    <t>Author:</t>
-  </si>
-  <si>
     <t>Pre-Mitigation Risk</t>
   </si>
   <si>
     <t>Post-Mitigation Risk</t>
+  </si>
+  <si>
+    <t>Organisation: Citrenz Group</t>
+  </si>
+  <si>
+    <t>Initiative, Project, and/or Engagement: Web conference for citrenz</t>
+  </si>
+  <si>
+    <t>Author: Ryan Wassell</t>
+  </si>
+  <si>
+    <t>Date: 8/03/2026</t>
+  </si>
+  <si>
+    <t>Sickness</t>
+  </si>
+  <si>
+    <t>Could miss out on client meetings, miss important information in class, lose time to work on project</t>
+  </si>
+  <si>
+    <t>Get enough sleep, stay hydrated, practice good hygiene</t>
+  </si>
+  <si>
+    <t>Work from home, email client/teachers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Being around other sick people, stress, poor diet, lack of sleep  </t>
+  </si>
+  <si>
+    <t>Scope Creep</t>
+  </si>
+  <si>
+    <t>Miss out on deadlines due to adding more features</t>
+  </si>
+  <si>
+    <t>Regularly talk to client</t>
+  </si>
+  <si>
+    <t>Do must have features first</t>
+  </si>
+  <si>
+    <t>Not sticking to project requirements, adding new features before must haves are finished</t>
+  </si>
+  <si>
+    <t>Poor Time Management</t>
+  </si>
+  <si>
+    <t>Rushed work, handing in work late</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stick to a timeline, try and do a little bit everyday </t>
+  </si>
+  <si>
+    <t>Ask for an extension</t>
+  </si>
+  <si>
+    <t>Procrastination, multiple projects</t>
+  </si>
+  <si>
+    <t>Data loss/corruption</t>
+  </si>
+  <si>
+    <t>Lost project progress</t>
+  </si>
+  <si>
+    <t>Back ups, Uploading to github</t>
+  </si>
+  <si>
+    <t>Restore from backups/github, ask for extra time if backsups/github doesn’t work</t>
+  </si>
+  <si>
+    <t>Software/Hardware Issues</t>
+  </si>
+  <si>
+    <t>Lack of specific technical logic for project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poor quality work, missing out on deadlines </t>
+  </si>
+  <si>
+    <t>Ask for help, search online resources</t>
+  </si>
+  <si>
+    <t>Ask for help, allocate extra time to learn content</t>
+  </si>
+  <si>
+    <t>New concepts needed for project</t>
   </si>
 </sst>
 </file>
@@ -491,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -539,6 +614,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -554,6 +632,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -834,7 +916,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
@@ -844,27 +926,27 @@
     </row>
     <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="D7" s="14" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="13"/>
       <c r="H7" s="15" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
@@ -872,22 +954,22 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="8"/>
       <c r="B8" s="19" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" s="20"/>
       <c r="D8" s="9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J8" s="11"/>
       <c r="K8" s="8"/>
@@ -896,192 +978,246 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="I9" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="J9" s="4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>0</v>
       </c>
       <c r="M9" s="18"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="102" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>1</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="3">
-        <v>0</v>
+      <c r="B10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="21">
+        <v>0.35</v>
       </c>
       <c r="E10" s="3">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" ref="F10:F29" si="0">D10*E10</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
+        <v>2.8</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="21">
+        <v>0.25</v>
+      </c>
+      <c r="I10" s="3">
+        <v>5</v>
+      </c>
       <c r="J10" s="3">
         <f t="shared" ref="J10:J29" si="1">H10*I10</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
+        <v>1.25</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="M10" s="16"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="102" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>2</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="3">
-        <v>0</v>
+      <c r="B11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="21">
+        <v>0.15</v>
       </c>
       <c r="E11" s="3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F11" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="3">
-        <v>0</v>
+        <v>0.75</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="21">
+        <v>0.05</v>
       </c>
       <c r="I11" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J11" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
+        <f>H11*I11</f>
+        <v>0.1</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="M11" s="16"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>3</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="3">
-        <v>0</v>
+      <c r="B12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="21">
+        <v>0.5</v>
       </c>
       <c r="E12" s="3">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="3">
-        <v>0</v>
+        <v>3.5</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" s="21">
+        <v>0.25</v>
       </c>
       <c r="I12" s="3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J12" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
+        <v>1.25</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="M12" s="16"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>4</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="3">
-        <v>0</v>
+      <c r="B13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="21">
+        <v>0.1</v>
       </c>
       <c r="E13" s="3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F13" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="3">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" s="21">
+        <v>0.05</v>
       </c>
       <c r="I13" s="3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J13" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
+        <v>0.25</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="M13" s="16"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>5</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="3">
-        <v>0</v>
+      <c r="B14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="21">
+        <v>0.3</v>
       </c>
       <c r="E14" s="3">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F14" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="3">
-        <v>0</v>
+        <v>2.4</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" s="21">
+        <v>0.2</v>
       </c>
       <c r="I14" s="3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J14" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="M14" s="16"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
@@ -1090,12 +1226,8 @@
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
-      <c r="D15" s="3">
-        <v>0</v>
-      </c>
-      <c r="E15" s="3">
-        <v>0</v>
-      </c>
+      <c r="D15" s="21"/>
+      <c r="E15" s="3"/>
       <c r="F15" s="3">
         <f t="shared" si="0"/>
         <v>0</v>

</xml_diff>